<commit_message>
added diagram stuff, weitere korrekturschleife halb durch (bis seite 21)
</commit_message>
<xml_diff>
--- a/Requirements.xlsx
+++ b/Requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://siemens-my.sharepoint.com/personal/malte-benedikt_schroeter_siemens_com/Documents/BA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3997" documentId="13_ncr:1_{BE626DFE-17E3-4385-820A-E055A2D8DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B75F60E-6674-4828-9D54-62824FE12247}"/>
+  <xr:revisionPtr revIDLastSave="4004" documentId="13_ncr:1_{BE626DFE-17E3-4385-820A-E055A2D8DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0262D64-1273-4F98-BCB8-0E10557AC108}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="5" xr2:uid="{9AFE01D9-9480-4035-82AC-131C794FF07E}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3160" uniqueCount="1035">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3161" uniqueCount="1036">
   <si>
     <t>ID</t>
   </si>
@@ -3344,10 +3344,13 @@
     <t>[Anpassung 06.08.2026] Nicht in den Katalog aufgenommen: Die Nachvollziehbarkeit von Änderungen an geschützten Geräteparametern (UC-12) wird nicht als Anforderung geführt. Die ID bleibt reserviert.</t>
   </si>
   <si>
-    <t>Kann man schreiben von Daten mit einer Registerabfrage validieren?</t>
-  </si>
-  <si>
-    <t>Thema  Polling-Geschwindigkeit?</t>
+    <t>In Kontakt mit EP Product Support (Stefan Baier, Sebastian Winklmann-Roehricht)</t>
+  </si>
+  <si>
+    <t>Arbeit: Analyse solider Anfang, mache ich bis zum Urlaub fertig</t>
+  </si>
+  <si>
+    <t>Objektmodell: bereits mit Andreas Ulmer im Kontakt, manche Dinge funktionieren noch nicht, teilweise liegt es am Gerät, das gilt es jetzt aber noch final herauszufinden</t>
   </si>
 </sst>
 </file>
@@ -3971,6 +3974,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>562904</xdr:colOff>
+      <xdr:row>109</xdr:row>
+      <xdr:rowOff>19638</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Grafik 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9677014A-30CC-6D7E-99DA-42FCB45BB090}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6162675" y="16573500"/>
+          <a:ext cx="6658904" cy="4210638"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -17140,6 +17187,11 @@
         <v>1034</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1035</v>
+      </c>
+    </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>560</v>

</xml_diff>

<commit_message>
Add new references to the bibliography for smart building applications and BMS data mapping
- Included articles by Balaji et al. (2018), Wang et al. (2018), Perumal et al. (2010), and Zhan et al. (2020) to enhance the literature review section.
- Ensured all entries are verified against publisher metadata via Crossref API.
- Added notes on the methodology for sourcing and verifying bibliographic information.
</commit_message>
<xml_diff>
--- a/Requirements.xlsx
+++ b/Requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://siemens-my.sharepoint.com/personal/malte-benedikt_schroeter_siemens_com/Documents/BA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4005" documentId="13_ncr:1_{BE626DFE-17E3-4385-820A-E055A2D8DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC2A6305-33B6-4086-8EC9-3F3D1F979EE5}"/>
+  <xr:revisionPtr revIDLastSave="4008" documentId="13_ncr:1_{BE626DFE-17E3-4385-820A-E055A2D8DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{862F0123-41EC-4C67-A1D9-0A64F92C0FC3}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="31530" yWindow="3030" windowWidth="21600" windowHeight="11295" xr2:uid="{9AFE01D9-9480-4035-82AC-131C794FF07E}"/>
+    <workbookView minimized="1" xWindow="5685" yWindow="4005" windowWidth="21600" windowHeight="11295" xr2:uid="{9AFE01D9-9480-4035-82AC-131C794FF07E}"/>
   </bookViews>
   <sheets>
     <sheet name="Funktional" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3161" uniqueCount="1036">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3162" uniqueCount="1037">
   <si>
     <t>ID</t>
   </si>
@@ -3350,7 +3350,10 @@
     <t>Objektmodell: bereits mit Andreas Ulmer im Kontakt, manche Dinge funktionieren noch nicht, teilweise liegt es am Gerät, das gilt es jetzt aber noch final herauszufinden</t>
   </si>
   <si>
-    <t>y</t>
+    <t xml:space="preserve">Anfrage elektronisches Schalten funktioniert mit </t>
+  </si>
+  <si>
+    <t>Die Kommunikation muss zyklisch erfolgen und Datenpunkte zyklisch übermitteln. Die Frequenz soll konfigurierbar sein.</t>
   </si>
 </sst>
 </file>
@@ -4018,6 +4021,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>113</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>44316</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>37784</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Grafik 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7DA5BCB-34E4-E4DF-D0DB-C4B4EE2EBFCD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6158962" y="21891356"/>
+          <a:ext cx="14460968" cy="2362530"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4371,12 +4418,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="C3" s="1"/>
     </row>
@@ -17166,7 +17213,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07379391-C6A2-4A97-9B7F-58688E513D59}">
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="92.42578125" customWidth="1"/>
@@ -17210,6 +17257,11 @@
     <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>1015</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
+        <v>1035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update bibliography entries in quellen.bib for accuracy and completeness
- Verified and corrected publication details for IEC standards, including titles, editions, and publication dates.
- Added notes regarding the verification of page numbers and publication details for various entries.
- Updated author and organization information for the IEC 62020 entry to reflect the German version.
- Included additional entries for oral communications with Siemens AG, specifying the context and format of the information provided.
</commit_message>
<xml_diff>
--- a/Requirements.xlsx
+++ b/Requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://siemens-my.sharepoint.com/personal/malte-benedikt_schroeter_siemens_com/Documents/BA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4546" documentId="13_ncr:1_{BE626DFE-17E3-4385-820A-E055A2D8DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B29399F-DBED-452F-96FA-4666E7F9FCBB}"/>
+  <xr:revisionPtr revIDLastSave="4549" documentId="13_ncr:1_{BE626DFE-17E3-4385-820A-E055A2D8DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C2374D3-BD48-4875-B39E-A71289549F97}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" firstSheet="5" activeTab="8" xr2:uid="{9AFE01D9-9480-4035-82AC-131C794FF07E}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="5" activeTab="6" xr2:uid="{9AFE01D9-9480-4035-82AC-131C794FF07E}"/>
   </bookViews>
   <sheets>
     <sheet name="Funktional" sheetId="1" r:id="rId1"/>
@@ -18166,7 +18166,7 @@
         <v>754</v>
       </c>
       <c r="E15" s="26">
-        <v>528</v>
+        <v>669</v>
       </c>
       <c r="F15" s="26" t="s">
         <v>229</v>
@@ -18201,7 +18201,7 @@
         <v>754</v>
       </c>
       <c r="E16" s="26">
-        <v>529</v>
+        <v>671</v>
       </c>
       <c r="F16" s="26" t="s">
         <v>230</v>
@@ -18236,7 +18236,7 @@
         <v>754</v>
       </c>
       <c r="E17" s="26">
-        <v>530</v>
+        <v>673</v>
       </c>
       <c r="F17" s="26" t="s">
         <v>231</v>
@@ -19125,7 +19125,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:K25" xr:uid="{215D1AA0-9FFC-4039-8385-BFD3A8114B33}"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Abhaken" prompt="Haken setzen, wenn der Datenpunkt in Desigo CC angelegt ist." sqref="A7:A25" xr:uid="{B3C75486-06C8-4D45-9126-EDECCD324AA8}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
@@ -22192,7 +22192,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:K71" xr:uid="{FB8EDA5B-3056-480A-AA43-F447F580627A}"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Abhaken" prompt="Haken setzen, wenn der Datenpunkt in Desigo CC angelegt ist." sqref="A7:A71" xr:uid="{18F9A785-CE63-4312-ADB5-134312DCB15D}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">

</xml_diff>